<commit_message>
Refactor: Integrate Snowflake Q1 growth analytics & AWS B partnership into LSEG Matrix
</commit_message>
<xml_diff>
--- a/M82_Sector_Rotation_Matrix.xlsx
+++ b/M82_Sector_Rotation_Matrix.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="B2:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,6 @@
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -537,7 +536,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -569,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="B3:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -579,8 +577,6 @@
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3">
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -784,42 +780,42 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Software - Application</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="C13" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>LEADING</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Estable</t>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Rally SNOW +40% / Contrato AWS $6B</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Alineacion</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Estable</t>
+      <c r="C14" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>LEADING</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Rally SNOW +40% / Contrato AWS $6B</t>
         </is>
       </c>
     </row>

</xml_diff>